<commit_message>
new version of script, changed the destination spreadsheet
</commit_message>
<xml_diff>
--- a/portfolio_allocations/VWCE_allocation.xlsx
+++ b/portfolio_allocations/VWCE_allocation.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Market Allocation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Allocation" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -475,14 +475,14 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.17764</v>
+        <v>0.16592</v>
       </c>
       <c r="F2" t="n">
-        <v>0.17352</v>
+        <v>0.16453</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -508,14 +508,14 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.07886</v>
+        <v>0.07721</v>
       </c>
       <c r="F3" t="n">
-        <v>0.07858</v>
+        <v>0.07682</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -541,14 +541,14 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1.6808</v>
+        <v>1.63761</v>
       </c>
       <c r="F4" t="n">
-        <v>1.68787</v>
+        <v>1.64462</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -574,14 +574,14 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.25757</v>
+        <v>0.24922</v>
       </c>
       <c r="F5" t="n">
-        <v>0.25349</v>
+        <v>0.24462</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -607,14 +607,14 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.5426</v>
+        <v>0.51391</v>
       </c>
       <c r="F6" t="n">
-        <v>0.53986</v>
+        <v>0.50997</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -640,14 +640,14 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3.15994</v>
+        <v>3.06937</v>
       </c>
       <c r="F7" t="n">
-        <v>3.15243</v>
+        <v>3.05889</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -673,14 +673,14 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2.1085</v>
+        <v>2.02423</v>
       </c>
       <c r="F8" t="n">
-        <v>2.11243</v>
+        <v>2.0261</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -706,14 +706,14 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.07771</v>
+        <v>0.07438</v>
       </c>
       <c r="F9" t="n">
-        <v>0.07507</v>
+        <v>0.07178</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>3.18372</v>
+        <v>2.99985</v>
       </c>
       <c r="F10" t="n">
-        <v>3.19845</v>
+        <v>3.02009</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -772,14 +772,14 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.0232</v>
+        <v>0.02006</v>
       </c>
       <c r="F11" t="n">
-        <v>0.02558</v>
+        <v>0.02198</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -805,14 +805,14 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.01441</v>
+        <v>0.01311</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0159</v>
+        <v>0.01501</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -838,14 +838,14 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1.9656</v>
+        <v>1.9301</v>
       </c>
       <c r="F13" t="n">
-        <v>1.96344</v>
+        <v>1.92633</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -871,14 +871,14 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.34835</v>
+        <v>0.34666</v>
       </c>
       <c r="F14" t="n">
-        <v>0.35</v>
+        <v>0.34866</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -904,14 +904,14 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.00494</v>
+        <v>0.0049</v>
       </c>
       <c r="F15" t="n">
-        <v>0.00725</v>
+        <v>0.00763</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -937,14 +937,14 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.85649</v>
+        <v>0.82364</v>
       </c>
       <c r="F16" t="n">
-        <v>0.85602</v>
+        <v>0.82465</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -970,14 +970,14 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.26774</v>
+        <v>0.27711</v>
       </c>
       <c r="F17" t="n">
-        <v>0.26452</v>
+        <v>0.27308</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1003,14 +1003,14 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2.18411</v>
+        <v>2.08118</v>
       </c>
       <c r="F18" t="n">
-        <v>2.19301</v>
+        <v>2.08973</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1036,14 +1036,14 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>3.53055</v>
+        <v>3.38025</v>
       </c>
       <c r="F19" t="n">
-        <v>3.42595</v>
+        <v>3.31933</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1069,14 +1069,14 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.07457999999999999</v>
+        <v>0.07360999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>0.07633</v>
+        <v>0.07531</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1102,14 +1102,14 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.52713</v>
+        <v>0.4962</v>
       </c>
       <c r="F21" t="n">
-        <v>0.52239</v>
+        <v>0.49414</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1135,14 +1135,14 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.04028</v>
+        <v>0.04529</v>
       </c>
       <c r="F22" t="n">
-        <v>0.04066</v>
+        <v>0.04533</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1168,14 +1168,14 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.10252</v>
+        <v>0.08482000000000001</v>
       </c>
       <c r="F23" t="n">
-        <v>0.10867</v>
+        <v>0.09075</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1201,14 +1201,14 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.08025</v>
+        <v>0.07887</v>
       </c>
       <c r="F24" t="n">
-        <v>0.07881000000000001</v>
+        <v>0.07779</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1234,14 +1234,14 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.3254</v>
+        <v>0.33934</v>
       </c>
       <c r="F25" t="n">
-        <v>0.32189</v>
+        <v>0.33579</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1267,14 +1267,14 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1.64123</v>
+        <v>1.6376</v>
       </c>
       <c r="F26" t="n">
-        <v>1.64538</v>
+        <v>1.63308</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1300,14 +1300,14 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.0105</v>
+        <v>0.0098</v>
       </c>
       <c r="F27" t="n">
-        <v>0.00765</v>
+        <v>0.00736</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1333,14 +1333,14 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.7839699999999999</v>
+        <v>0.79399</v>
       </c>
       <c r="F28" t="n">
-        <v>0.78498</v>
+        <v>0.79414</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1366,14 +1366,14 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>5.8715</v>
+        <v>5.81311</v>
       </c>
       <c r="F29" t="n">
-        <v>5.87375</v>
+        <v>5.81391</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1399,14 +1399,14 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1.80392</v>
+        <v>2.26177</v>
       </c>
       <c r="F30" t="n">
-        <v>1.8122</v>
+        <v>2.26601</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1432,14 +1432,14 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.07661999999999999</v>
+        <v>0.07019</v>
       </c>
       <c r="F31" t="n">
-        <v>0.07838000000000001</v>
+        <v>0.07382</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1465,14 +1465,14 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.25207</v>
+        <v>0.23482</v>
       </c>
       <c r="F32" t="n">
-        <v>0.25689</v>
+        <v>0.23867</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1498,14 +1498,14 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.17576</v>
+        <v>0.16693</v>
       </c>
       <c r="F33" t="n">
-        <v>0.17738</v>
+        <v>0.16777</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1531,14 +1531,14 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>1.09253</v>
+        <v>1.09585</v>
       </c>
       <c r="F34" t="n">
-        <v>1.09092</v>
+        <v>1.09151</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1564,14 +1564,14 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0.17072</v>
+        <v>0.15231</v>
       </c>
       <c r="F35" t="n">
-        <v>0.16984</v>
+        <v>0.15168</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1597,14 +1597,14 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0.05154</v>
+        <v>0.04946</v>
       </c>
       <c r="F36" t="n">
-        <v>0.05085</v>
+        <v>0.0484</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1630,11 +1630,11 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.00022</v>
+        <v>0.00405</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1660,14 +1660,14 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.04775</v>
+        <v>0.04247</v>
       </c>
       <c r="F38" t="n">
-        <v>0.04743</v>
+        <v>0.04201</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1693,14 +1693,14 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.10484</v>
+        <v>0.1021</v>
       </c>
       <c r="F39" t="n">
-        <v>0.10834</v>
+        <v>0.10598</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1726,14 +1726,14 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.04978</v>
+        <v>0.04693</v>
       </c>
       <c r="F40" t="n">
-        <v>0.04994</v>
+        <v>0.04708</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1759,14 +1759,14 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.07586</v>
+        <v>0.07174</v>
       </c>
       <c r="F41" t="n">
-        <v>0.07306</v>
+        <v>0.06845</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1792,14 +1792,14 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.01411</v>
+        <v>0.01318</v>
       </c>
       <c r="F42" t="n">
-        <v>0.01449</v>
+        <v>0.01349</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1855,14 +1855,14 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.3862</v>
+        <v>0.34777</v>
       </c>
       <c r="F44" t="n">
-        <v>0.38521</v>
+        <v>0.34705</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1888,14 +1888,14 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.75329</v>
+        <v>0.73372</v>
       </c>
       <c r="F45" t="n">
-        <v>0.75061</v>
+        <v>0.73046</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1921,14 +1921,14 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.37859</v>
+        <v>0.35202</v>
       </c>
       <c r="F46" t="n">
-        <v>0.36587</v>
+        <v>0.33886</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1954,14 +1954,14 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.16438</v>
+        <v>0.15317</v>
       </c>
       <c r="F47" t="n">
-        <v>0.16992</v>
+        <v>0.15876</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -1987,14 +1987,14 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.10325</v>
+        <v>0.10331</v>
       </c>
       <c r="F48" t="n">
-        <v>0.11027</v>
+        <v>0.11075</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -2020,14 +2020,14 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>2.60744</v>
+        <v>2.95987</v>
       </c>
       <c r="F49" t="n">
-        <v>2.61146</v>
+        <v>2.98162</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -2053,14 +2053,14 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>61.33677</v>
+        <v>61.57311</v>
       </c>
       <c r="F50" t="n">
-        <v>61.40943</v>
+        <v>61.60314</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
@@ -2086,14 +2086,14 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>0.43427</v>
+        <v>0.40389</v>
       </c>
       <c r="F51" t="n">
-        <v>0.43366</v>
+        <v>0.40308</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>

</xml_diff>